<commit_message>
Commit registry rename and panel updates
</commit_message>
<xml_diff>
--- a/MH_Registry/Config.xlsx
+++ b/MH_Registry/Config.xlsx
@@ -3782,6 +3782,622 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cánh Dưới</t>
+        </is>
+      </c>
+      <c r="B2"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cánh Lật</t>
+        </is>
+      </c>
+      <c r="B3"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cánh Phải</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cánh Trái</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cánh Trên</t>
+        </is>
+      </c>
+      <c r="B6"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chặn Cánh</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CNC Họa Tiết</t>
+        </is>
+      </c>
+      <c r="B8"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CNK</t>
+        </is>
+      </c>
+      <c r="B9"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đầu Giường</t>
+        </is>
+      </c>
+      <c r="B10"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đáy</t>
+        </is>
+      </c>
+      <c r="B11"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đáy Hộc</t>
+        </is>
+      </c>
+      <c r="B12"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đáy Hộc NK</t>
+        </is>
+      </c>
+      <c r="B13"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đợt Cố Định</t>
+        </is>
+      </c>
+      <c r="B14"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đợt Di Động</t>
+        </is>
+      </c>
+      <c r="B15"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đuôi Giường</t>
+        </is>
+      </c>
+      <c r="B16"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dưỡng</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">11</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dưỡng Uốn</t>
+        </is>
+      </c>
+      <c r="B18"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Giằng</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Giằng Bệ Chân</t>
+        </is>
+      </c>
+      <c r="B20"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Giằng Sau</t>
+        </is>
+      </c>
+      <c r="B21"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Giằng Trước</t>
+        </is>
+      </c>
+      <c r="B22"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gương bỉ dày 5mm</t>
+        </is>
+      </c>
+      <c r="B23"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hậu</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">44</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hộc - Đáy</t>
+        </is>
+      </c>
+      <c r="B25"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hộc - Thành Phải</t>
+        </is>
+      </c>
+      <c r="B26"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hộc - Thành Sau</t>
+        </is>
+      </c>
+      <c r="B27"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hộc - Thành Trái</t>
+        </is>
+      </c>
+      <c r="B28"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hộc - Thành Trước</t>
+        </is>
+      </c>
+      <c r="B29"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hộc NK</t>
+        </is>
+      </c>
+      <c r="B30"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hông Giữa</t>
+        </is>
+      </c>
+      <c r="B31"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hông Lộ</t>
+        </is>
+      </c>
+      <c r="B32"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hông Phải</t>
+        </is>
+      </c>
+      <c r="B33"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hông Trái</t>
+        </is>
+      </c>
+      <c r="B34"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Len Chân</t>
+        </is>
+      </c>
+      <c r="B35"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Len Chân Trước</t>
+        </is>
+      </c>
+      <c r="B36"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mặt Bàn</t>
+        </is>
+      </c>
+      <c r="B37"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mặt Bệ Chân</t>
+        </is>
+      </c>
+      <c r="B38"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mặt Len Chân</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">123</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mặt NK</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nan</t>
+        </is>
+      </c>
+      <c r="B41"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nền Tấm Fix</t>
+        </is>
+      </c>
+      <c r="B42"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nẹp</t>
+        </is>
+      </c>
+      <c r="B43"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nẹp Bù</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nẹp Tăng Dày</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">12</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nóc</t>
+        </is>
+      </c>
+      <c r="B46"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nóc Hộc</t>
+        </is>
+      </c>
+      <c r="B47"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Phào Nóc</t>
+        </is>
+      </c>
+      <c r="B48"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tấm Fix</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">111</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tấm inox</t>
+        </is>
+      </c>
+      <c r="B50"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tấm Mặt</t>
+        </is>
+      </c>
+      <c r="B51"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tấm Nền</t>
+        </is>
+      </c>
+      <c r="B52"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tấm Uốn</t>
+        </is>
+      </c>
+      <c r="B53"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tấm Uốn Cong</t>
+        </is>
+      </c>
+      <c r="B54"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tạo Dày Hông Phải</t>
+        </is>
+      </c>
+      <c r="B55"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tạo Dày Hông Trái</t>
+        </is>
+      </c>
+      <c r="B56"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tay Nắm</t>
+        </is>
+      </c>
+      <c r="B57"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Thanh Bản Lề</t>
+        </is>
+      </c>
+      <c r="B58"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vách</t>
+        </is>
+      </c>
+      <c r="B59"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vai Giường</t>
+        </is>
+      </c>
+      <c r="B60"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Viền Cánh</t>
+        </is>
+      </c>
+      <c r="B61"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Viền Mặt Bàn</t>
+        </is>
+      </c>
+      <c r="B62"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Xương</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">123</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Xương Nẹp</t>
+        </is>
+      </c>
+      <c r="B64"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Khuôn Cửa</t>
+        </is>
+      </c>
+      <c r="B65"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hông</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hậu Lộ</t>
+        </is>
+      </c>
+      <c r="B67"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gương</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">111</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kính</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">222</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Inox</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">333</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore(app): checkpoint plugin state and add Module Studio performance diagnosis
- Add MH_Module_Studio/PERFORMANCE_DIAGNOSIS.md: measured breakdown of the
  T1 options-update slowdown. Dominant cost is the GVL yield in
  UpdateWork.compute: sleep(0.001) actually takes ~15.6 ms in this process
  (764-738 yields = ~11 s of a 11-16 s job, process CPU only ~1 s).
  A/B on real work: sleep(0.001) 7.6-10.2x slower than the same work with
  no yield; sleep(0) and Thread.pass cost ~0.02 ms per yield.
  Secondary: repeated full-rule validate/copy/serialize (~1 s CPU).
- Include pending work across MH_CAD2Module, MH_Module_Studio and the other
  plugin families (228 new files, 160 modified, 1 deleted).
</commit_message>
<xml_diff>
--- a/MH_Registry/Config.xlsx
+++ b/MH_Registry/Config.xlsx
@@ -11,12 +11,10 @@
     <sheet name="ma_thickness" sheetId="7" r:id="rId7"/>
     <sheet name="ma_detail_aliases" sheetId="8" r:id="rId8"/>
     <sheet name="ma_tag_materials" sheetId="9" r:id="rId9"/>
-    <sheet name="ma_valid" sheetId="10" r:id="rId10"/>
-    <sheet name="ma_invalid" sheetId="11" r:id="rId11"/>
-    <sheet name="ma_column_aliases" sheetId="12" r:id="rId12"/>
-    <sheet name="ma_surface_face_rules" sheetId="13" r:id="rId13"/>
-    <sheet name="panel_defaults" sheetId="14" r:id="rId14"/>
-    <sheet name="dc_thickness_options_project" sheetId="15" r:id="rId15"/>
+    <sheet name="ma_column_aliases" sheetId="10" r:id="rId10"/>
+    <sheet name="ma_surface_face_rules" sheetId="11" r:id="rId11"/>
+    <sheet name="panel_defaults" sheetId="12" r:id="rId12"/>
+    <sheet name="dc_thickness_options_project" sheetId="13" r:id="rId13"/>
   </sheets>
 </workbook>
 </file>
@@ -164,708 +162,322 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">material</t>
+          <t xml:space="preserve">internal_name</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t xml:space="preserve">thickness</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">actual_thickness</t>
+          <t xml:space="preserve">alias</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GONHUA</t>
+          <t xml:space="preserve">Ma_SP</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">8</t>
-        </is>
-      </c>
-      <c r="C2"/>
+          <t xml:space="preserve">Ma_SP</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">GONHUA</t>
+          <t xml:space="preserve">Ma_SP</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">12</t>
-        </is>
-      </c>
-      <c r="C3"/>
+          <t xml:space="preserve">Mã SP</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">GONHUA</t>
+          <t xml:space="preserve">Ma_SP</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">17</t>
-        </is>
-      </c>
-      <c r="C4"/>
+          <t xml:space="preserve">Ma SP</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDFCA</t>
+          <t xml:space="preserve">Ma_SP</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">8</t>
-        </is>
-      </c>
-      <c r="C5"/>
+          <t xml:space="preserve">Mã sp</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDFCA</t>
+          <t xml:space="preserve">Ma_SP</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">12</t>
-        </is>
-      </c>
-      <c r="C6"/>
+          <t xml:space="preserve">MÃ£ sáº£n pháº©m</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDFCA</t>
+          <t xml:space="preserve">Ma_SP</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">15</t>
-        </is>
-      </c>
-      <c r="C7"/>
+          <t xml:space="preserve">Ma san pham</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDFCA</t>
+          <t xml:space="preserve">Ma_SP</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">17</t>
-        </is>
-      </c>
-      <c r="C8"/>
+          <t xml:space="preserve">Product Code</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDFCA.AC</t>
+          <t xml:space="preserve">Ma_SP</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">9</t>
-        </is>
-      </c>
-      <c r="C9"/>
+          <t xml:space="preserve">SP</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDFCA.AC</t>
+          <t xml:space="preserve">Ma_vat_lieu</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">12</t>
-        </is>
-      </c>
-      <c r="C10"/>
+          <t xml:space="preserve">Ma_vat_lieu</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDFCA.AC</t>
+          <t xml:space="preserve">Ma_vat_lieu</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">17</t>
-        </is>
-      </c>
-      <c r="C11"/>
+          <t xml:space="preserve">Ma vat lieu</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDFCA.AC.LK</t>
+          <t xml:space="preserve">Ma_vat_lieu</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">9</t>
-        </is>
-      </c>
-      <c r="C12"/>
+          <t xml:space="preserve">Mã vật liệu</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDFCA.AC.LK</t>
+          <t xml:space="preserve">Ma_vat_lieu</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">12</t>
-        </is>
-      </c>
-      <c r="C13"/>
+          <t xml:space="preserve">Mã Vật Liệu</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDFCA.AC.LK</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">19</t>
-        </is>
-      </c>
-      <c r="C14"/>
+          <t xml:space="preserve">Ma_vat_lieu</t>
+        </is>
+      </c>
+      <c r="B14"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">MDFCA</t>
+          <t xml:space="preserve">Ma_vat_lieu</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">17</t>
-        </is>
-      </c>
-      <c r="C15"/>
+          <t xml:space="preserve">Ma VL</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">PICOMAT</t>
+          <t xml:space="preserve">Ma_vat_lieu</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">8</t>
-        </is>
-      </c>
-      <c r="C16"/>
+          <t xml:space="preserve">Material Code</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">PICOMAT</t>
+          <t xml:space="preserve">Ma_vat_lieu</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">18</t>
-        </is>
-      </c>
-      <c r="C17"/>
+          <t xml:space="preserve">Material</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">PLY</t>
+          <t xml:space="preserve">Ma_vat_lieu</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">9</t>
-        </is>
-      </c>
-      <c r="C18"/>
+          <t xml:space="preserve">VL</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">PLY</t>
+          <t xml:space="preserve">Ten_chi_tiet</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">12</t>
-        </is>
-      </c>
-      <c r="C19"/>
+          <t xml:space="preserve">Ten_chi_tiet</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">PLY</t>
+          <t xml:space="preserve">Ten_chi_tiet</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">17</t>
-        </is>
-      </c>
-      <c r="C20"/>
+          <t xml:space="preserve">Tên Chi Tiết</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">PLY.AC</t>
+          <t xml:space="preserve">Ten_chi_tiet</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">9</t>
-        </is>
-      </c>
-      <c r="C21"/>
+          <t xml:space="preserve">Tên chi tiết</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">PLY.AC</t>
+          <t xml:space="preserve">Ten_chi_tiet</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">12</t>
-        </is>
-      </c>
-      <c r="C22"/>
+          <t xml:space="preserve">TenCT</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">PLY.AC</t>
+          <t xml:space="preserve">Ten_chi_tiet</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">17</t>
-        </is>
-      </c>
-      <c r="C23"/>
+          <t xml:space="preserve">Chi tiáº¿t</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">PLY.AC.LK</t>
+          <t xml:space="preserve">Ten_chi_tiet</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">9</t>
-        </is>
-      </c>
-      <c r="C24"/>
+          <t xml:space="preserve">Chi tiet</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">PLY.AC.LK</t>
+          <t xml:space="preserve">Ten_chi_tiet</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">12</t>
-        </is>
-      </c>
-      <c r="C25"/>
+          <t xml:space="preserve">Detail Name</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">PLY.AC.LK</t>
+          <t xml:space="preserve">Ten_chi_tiet</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">19</t>
-        </is>
-      </c>
-      <c r="C26"/>
+          <t xml:space="preserve">Detail</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">PLY.AC.VER</t>
+          <t xml:space="preserve">Ten_chi_tiet</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">12</t>
-        </is>
-      </c>
-      <c r="C27"/>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PLY.AC.VER</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">18</t>
-        </is>
-      </c>
-      <c r="C28"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PLY.AC.VERKT</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">9</t>
-        </is>
-      </c>
-      <c r="C29"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PLY.AC.VERKT</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">12</t>
-        </is>
-      </c>
-      <c r="C30"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PLY.AC.VERKT</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">18</t>
-        </is>
-      </c>
-      <c r="C31"/>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PLY.AC.VERSOI</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">9</t>
-        </is>
-      </c>
-      <c r="C32"/>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PLY.AC.VERSOI</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">12</t>
-        </is>
-      </c>
-      <c r="C33"/>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PLY.AC.VERSOI</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">18</t>
-        </is>
-      </c>
-      <c r="C34"/>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PLY.VER</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">9</t>
-        </is>
-      </c>
-      <c r="C35"/>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PLY.VER</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">12</t>
-        </is>
-      </c>
-      <c r="C36"/>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PLY.VER</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">18</t>
-        </is>
-      </c>
-      <c r="C37"/>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WPB</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6</t>
-        </is>
-      </c>
-      <c r="C38"/>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WPB</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8</t>
-        </is>
-      </c>
-      <c r="C39"/>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WPB</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10</t>
-        </is>
-      </c>
-      <c r="C40"/>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WPB</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">12</t>
-        </is>
-      </c>
-      <c r="C41"/>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WPB</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">15</t>
-        </is>
-      </c>
-      <c r="C42"/>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WPB</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">17</t>
-        </is>
-      </c>
-      <c r="C43"/>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WPB.LK</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">19</t>
-        </is>
-      </c>
-      <c r="C44"/>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GOSOI</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20</t>
-        </is>
-      </c>
-      <c r="C45"/>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GOSOI</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">26</t>
-        </is>
-      </c>
-      <c r="C46"/>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GOSOI</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">38</t>
-        </is>
-      </c>
-      <c r="C47"/>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GOSOI</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">50</t>
-        </is>
-      </c>
-      <c r="C48"/>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TANBI</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">26</t>
-        </is>
-      </c>
-      <c r="C49"/>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TANBI</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">30</t>
-        </is>
-      </c>
-      <c r="C50"/>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TANBI</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">32</t>
-        </is>
-      </c>
-      <c r="C51"/>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TANBI</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">38</t>
-        </is>
-      </c>
-      <c r="C52"/>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TANBI</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">40</t>
-        </is>
-      </c>
-      <c r="C53"/>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TANBI</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">50</t>
-        </is>
-      </c>
-      <c r="C54"/>
+          <t xml:space="preserve">TÃªn CT</t>
+        </is>
+      </c>
     </row>
   </sheetData>
 </worksheet>
@@ -877,12 +489,84 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">material</t>
+          <t xml:space="preserve">enabled</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t xml:space="preserve">thickness</t>
+          <t xml:space="preserve">surface_tokens</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">max_one_side_thickness</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one_side_suffix</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">two_side_details</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">two_side_suffix</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">default_suffix</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">finish_suffix_overrides</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LAM,LAMINATE,LK,VENE,VER</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">.1M</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đợt,Đợt Cố Định,Hông Giữa,Cánh,Pano Cánh,Cánh Trái,Cánh Phải,Chặn Cánh,Mặt NK,Hộc - Thành Phải,Hộc - Thành Trái,Hộc - Thành Trước,Hộc - Thành Sau,Đình,Mặt Bàn,Hông Lộ</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">.2M</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">.1M</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LK:.1M-BCT,.2M;LL:.1M-BCT,.2M</t>
         </is>
       </c>
     </row>
@@ -896,320 +580,17 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">internal_name</t>
+          <t xml:space="preserve">tool</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t xml:space="preserve">alias</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ma_SP</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ma_SP</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ma_SP</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Mã SP</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ma_SP</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ma SP</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ma_SP</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Mã sp</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ma_SP</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MÃ£ sáº£n pháº©m</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ma_SP</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ma san pham</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ma_SP</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Product Code</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ma_SP</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SP</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ma_vat_lieu</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ma_vat_lieu</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ma_vat_lieu</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ma vat lieu</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ma_vat_lieu</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Mã vật liệu</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ma_vat_lieu</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Mã Vật Liệu</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ma_vat_lieu</t>
-        </is>
-      </c>
-      <c r="B14"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ma_vat_lieu</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ma VL</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ma_vat_lieu</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Material Code</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ma_vat_lieu</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Material</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ma_vat_lieu</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">VL</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ten_chi_tiet</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ten_chi_tiet</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ten_chi_tiet</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tên Chi Tiết</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ten_chi_tiet</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tên chi tiết</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ten_chi_tiet</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TenCT</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ten_chi_tiet</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Chi tiáº¿t</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ten_chi_tiet</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Chi tiet</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ten_chi_tiet</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Detail Name</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ten_chi_tiet</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Detail</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ten_chi_tiet</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TÃªn CT</t>
+          <t xml:space="preserve">key</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">value</t>
         </is>
       </c>
     </row>
@@ -1223,121 +604,6 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">enabled</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">surface_tokens</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">max_one_side_thickness</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">one_side_suffix</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">two_side_details</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">two_side_suffix</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">default_suffix</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">finish_suffix_overrides</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LAM,LAMINATE,LK,VENE,VER</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">9</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">.1M</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Đợt,Đợt Cố Định,Hông Giữa,Cánh,Pano Cánh,Cánh Trái,Cánh Phải,Chặn Cánh,Mặt NK,Hộc - Thành Phải,Hộc - Thành Trái,Hộc - Thành Trước,Hộc - Thành Sau,Đình,Mặt Bàn,Hông Lộ</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">.2M</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">.1M</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LK:.1M-BCT,.2M;LL:.1M-BCT,.2M</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tool</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">key</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">value</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
           <t xml:space="preserve">material_type</t>
         </is>
       </c>
@@ -4813,34 +4079,34 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">An Cường</t>
+          <t xml:space="preserve">WPB</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">AC</t>
+          <t xml:space="preserve">WPB</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">nha_cung_cap</t>
+          <t xml:space="preserve">chat_lieu</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Panel</t>
+          <t xml:space="preserve">An Cường</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">PANEL</t>
+          <t xml:space="preserve">AC</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -4857,12 +4123,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">DONGWA</t>
+          <t xml:space="preserve">Panel</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">DONGWA</t>
+          <t xml:space="preserve">PANEL</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -4901,34 +4167,34 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Veneer</t>
+          <t xml:space="preserve">Dongwha</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">VER</t>
+          <t xml:space="preserve">DW</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">be_mat</t>
+          <t xml:space="preserve">nha_cung_cap</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Veneer kỹ thuật</t>
+          <t xml:space="preserve">Veneer</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERKT</t>
+          <t xml:space="preserve">VER</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -4945,12 +4211,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">VENEER KỸ THUẬT SỒI</t>
+          <t xml:space="preserve">Veneer kỹ thuật</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERKTSOI</t>
+          <t xml:space="preserve">VERKT</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -4967,12 +4233,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Veneer sồi</t>
+          <t xml:space="preserve">VENEER KỸ THUẬT SỒI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERSOI</t>
+          <t xml:space="preserve">VERKTSOI</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -4989,12 +4255,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Laminate</t>
+          <t xml:space="preserve">Veneer sồi</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">LK</t>
+          <t xml:space="preserve">VERSOI</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -5011,12 +4277,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sơn</t>
+          <t xml:space="preserve">Laminate</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">SON</t>
+          <t xml:space="preserve">LAM</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -5033,20 +4299,42 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t xml:space="preserve">Sơn</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SON</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">be_mat</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t xml:space="preserve">Melamine</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MS</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEL</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
         <is>
           <t xml:space="preserve">be_mat</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t xml:space="preserve">3</t>
         </is>

</xml_diff>